<commit_message>
fix(attendance): default missing employee checkouts to 7 PM and repair historical records
</commit_message>
<xml_diff>
--- a/HRMS_Project_Management.xlsx
+++ b/HRMS_Project_Management.xlsx
@@ -439,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1529,9 +1529,29 @@
         <v>* [COMPLETED] TSK-EMP-015 (Redesign Employee Profile Page to Match Executive Design Mockup): Overhauled the Employee Profile page to match the executive design mockup. Added breadcrumb navigation, More Actions dropdown, warm golden bronze Chat button linking to Google Chat, hero card with dark navy avatar, SSG employee code chip, bold name, ACTIVE pill, subtitle, inspirational quote, 3-column stats with dynamic Years With Us, 4-column contact strip, floating pill navigation tabs with Lucide icons, and 2x2 overview details cards grid with Edit buttons and alternating zebra-striped rows.</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="2" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B55" s="2" t="str">
+        <v>TSK-ATT-028</v>
+      </c>
+      <c r="C55" s="2" t="str">
+        <v>Default missing employee checkouts to 7:00 PM and repair historical records</v>
+      </c>
+      <c r="D55" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="E55" s="2" t="str">
+        <v>Resolved an issue where missing employee checkouts artificially received a fake 1-minute checkout timestamp (e.g. 10:39 AM for a 10:38 AM check-in) with 1m worked duration and Half Day status. Updated the daily automated finalization scheduler and manual finalize endpoint to assign 7:00 PM IST (19:00) as default checkout time for uncompleted checkouts (or preserve later desktop activity timestamps if present). Added startup repair fixIrrelevantCheckouts() to correct past affected records.</v>
+      </c>
+      <c r="F55" s="2" t="str">
+        <v>* [COMPLETED] TSK-ATT-028 (Default missing employee checkouts to 7:00 PM and repair historical records): Resolved an issue where missing employee checkouts artificially received a fake 1-minute checkout timestamp (e.g. 10:39 AM for a 10:38 AM check-in) with 1m worked duration and Half Day status. Updated the daily automated finalization scheduler and manual finalize endpoint to assign 7:00 PM IST (19:00) as default checkout time for uncompleted checkouts (or preserve later desktop activity timestamps if present). Added startup repair fixIrrelevantCheckouts() to correct past affected records.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F55"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2463,7 +2483,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W74"/>
+  <dimension ref="A1:W75"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -7744,9 +7764,80 @@
         <v>Overhauled the Executive Dashboard UI to match Figma reference mockup and completed full login page visual redesign. Redesigned Employee Profile page to match executive design mockup with breadcrumb header, More Actions dropdown, golden bronze Chat button, hero card with dark navy avatar, SSG employee code chip, bold name, ACTIVE pill, subtitle, quote, 3-column stats with dynamic Years With Us, 4-column contact strip, floating pill navigation tabs with Lucide icons, and 2x2 overview details cards grid with Edit buttons and alternating zebra-striped rows.</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="2" t="str">
+        <v>2026-09-24</v>
+      </c>
+      <c r="B75" s="2" t="str">
+        <v>Fullstack Team</v>
+      </c>
+      <c r="C75" s="2" t="str">
+        <v>HRMS</v>
+      </c>
+      <c r="D75" s="2" t="str">
+        <v>Sprint 4</v>
+      </c>
+      <c r="E75" s="2" t="str">
+        <v>Desktop Client / Web Dashboard</v>
+      </c>
+      <c r="F75" s="2" t="str">
+        <v>Attendance</v>
+      </c>
+      <c r="G75" s="2" t="str">
+        <v>Flexible Breaks, Penalties &amp; Agent Robustness</v>
+      </c>
+      <c r="H75" s="2" t="str">
+        <v>TSK-ATT-028</v>
+      </c>
+      <c r="I75" s="2" t="str">
+        <v>Implement Quota-Based Flexible Breaks, Penalties &amp; Desktop Agent Robustness</v>
+      </c>
+      <c r="J75" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="K75" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="L75" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="M75" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="N75" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="O75" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+      <c r="P75" s="2">
+        <v>6</v>
+      </c>
+      <c r="Q75" s="2">
+        <v>2</v>
+      </c>
+      <c r="R75" s="2" t="str">
+        <v>100%</v>
+      </c>
+      <c r="S75" s="2" t="str">
+        <v>COMPLETED</v>
+      </c>
+      <c r="T75" s="2" t="str">
+        <v>None</v>
+      </c>
+      <c r="U75" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="V75" s="2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="W75" s="2" t="str">
+        <v>Investigated and resolved the irrelevant checkout time issue on employee attendance records. Updated backend scheduler and finalization routes to assign 7:00 PM IST (19:00) when an employee does not check out manually, calculate accurate worked hours, and assign Present status. Implemented a startup repair function fixIrrelevantCheckouts() to correct past corrupted records.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W75"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>